<commit_message>
options bug fix in day3
</commit_message>
<xml_diff>
--- a/data/questions_2025_day3.xlsx
+++ b/data/questions_2025_day3.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="247">
   <si>
     <t>Energy consumption per unit of GDP is called as:</t>
   </si>
@@ -36,9 +36,6 @@
     <t xml:space="preserve">None </t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
     <t>Star rating is a part of ______ programme of BEE</t>
   </si>
   <si>
@@ -51,9 +48,6 @@
     <t>S&amp;L</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
     <t xml:space="preserve">As per IEGC (latest amendment) “frequency band” in Hz is </t>
   </si>
   <si>
@@ -69,9 +63,6 @@
     <t>49.5 – 50.2</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
     <t>Action for non-compliance of IEGC  may be taken by</t>
   </si>
   <si>
@@ -85,9 +76,6 @@
   </si>
   <si>
     <t>Central Electricity Regulatory Commission(CERC) on report by any person or suo-motu</t>
-  </si>
-  <si>
-    <t>D</t>
   </si>
   <si>
     <t xml:space="preserve"> A part of the grid can be deliberately isolated from the rest of the National/Regional grid, only</t>
@@ -1024,7 +1012,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1059,7 +1047,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1258,30 +1246,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>245</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>
@@ -1298,246 +1286,246 @@
       <c r="F2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="6" t="s">
-        <v>5</v>
+      <c r="G2" s="6">
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>8</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>9</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="8" t="s">
-        <v>10</v>
+      <c r="G3" s="8">
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>16</v>
+      <c r="G4" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="75" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>22</v>
+      <c r="G5" s="8">
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>22</v>
+      <c r="G6" s="8">
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="150" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="F7" s="32" t="s">
-        <v>235</v>
-      </c>
-      <c r="G7" s="25" t="s">
-        <v>22</v>
+        <v>231</v>
+      </c>
+      <c r="G7" s="25">
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="75" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>5</v>
+      <c r="G8" s="8">
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>10</v>
+        <v>225</v>
+      </c>
+      <c r="G9" s="8">
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="75" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>16</v>
+        <v>34</v>
+      </c>
+      <c r="G10" s="8">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="75" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>5</v>
+        <v>34</v>
+      </c>
+      <c r="G11" s="8">
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B12" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>5</v>
+      <c r="G12" s="10">
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C13" s="11">
         <v>0.02</v>
@@ -1551,16 +1539,16 @@
       <c r="F13" s="11">
         <v>0.05</v>
       </c>
-      <c r="G13" s="10" t="s">
-        <v>10</v>
+      <c r="G13" s="10">
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C14" s="12">
         <v>1.4999999999999999E-2</v>
@@ -1574,177 +1562,177 @@
       <c r="F14" s="12">
         <v>0.05</v>
       </c>
-      <c r="G14" s="10" t="s">
-        <v>22</v>
+      <c r="G14" s="10">
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>5</v>
+      <c r="G15" s="10">
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="45" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B16" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>5</v>
+      <c r="G16" s="10">
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="75" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>5</v>
+        <v>55</v>
+      </c>
+      <c r="G17" s="10">
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F18" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="G18" s="13" t="s">
-        <v>5</v>
+      <c r="G18" s="13">
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B19" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F19" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="F19" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="G19" s="17" t="s">
-        <v>5</v>
+      <c r="G19" s="17">
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="45" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B20" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="F20" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="F20" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="G20" s="17" t="s">
-        <v>22</v>
+      <c r="G20" s="17">
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B21" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="F21" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="C21" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="F21" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="G21" s="17" t="s">
-        <v>22</v>
+      <c r="G21" s="17">
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C22" s="18">
         <v>0.1</v>
@@ -1758,108 +1746,108 @@
       <c r="F22" s="19">
         <v>0.08</v>
       </c>
-      <c r="G22" s="17" t="s">
-        <v>22</v>
+      <c r="G22" s="17">
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B23" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="F23" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="G23" s="10" t="s">
-        <v>5</v>
+      <c r="G23" s="10">
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B24" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="F24" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G24" s="10" t="s">
-        <v>22</v>
+      <c r="G24" s="10">
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G25" s="10" t="s">
-        <v>16</v>
+        <v>86</v>
+      </c>
+      <c r="G25" s="10">
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B26" s="20" t="s">
+        <v>226</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>228</v>
+      </c>
+      <c r="E26" s="21" t="s">
+        <v>229</v>
+      </c>
+      <c r="F26" s="21" t="s">
         <v>230</v>
       </c>
-      <c r="C26" s="21" t="s">
-        <v>231</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>232</v>
-      </c>
-      <c r="E26" s="21" t="s">
-        <v>233</v>
-      </c>
-      <c r="F26" s="21" t="s">
-        <v>234</v>
-      </c>
-      <c r="G26" s="22" t="s">
-        <v>16</v>
+      <c r="G26" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C27" s="5">
         <v>6.06</v>
@@ -1873,269 +1861,269 @@
       <c r="F27" s="5">
         <v>2.3490000000000002</v>
       </c>
-      <c r="G27" s="23" t="s">
-        <v>10</v>
+      <c r="G27" s="23">
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="45" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B28" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F28" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C28" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G28" s="23" t="s">
-        <v>5</v>
+      <c r="G28" s="23">
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B29" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="F29" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C29" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="G29" s="23" t="s">
-        <v>10</v>
+      <c r="G29" s="23">
+        <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B30" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="G30" s="23" t="s">
-        <v>5</v>
+      <c r="G30" s="23">
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B31" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="F31" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C31" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="G31" s="23" t="s">
-        <v>5</v>
+      <c r="G31" s="23">
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="45" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B32" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="F32" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C32" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="G32" s="23" t="s">
-        <v>16</v>
+      <c r="G32" s="23">
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="45" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B33" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F33" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="G33" s="23" t="s">
-        <v>5</v>
+      <c r="G33" s="23">
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="75" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B34" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="F34" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C34" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="G34" s="23" t="s">
-        <v>10</v>
+      <c r="G34" s="23">
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B35" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F35" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="C35" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="G35" s="23" t="s">
-        <v>10</v>
+      <c r="G35" s="23">
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B36" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="F36" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="C36" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="G36" s="23" t="s">
-        <v>5</v>
+      <c r="G36" s="23">
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B37" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F37" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C37" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="G37" s="23" t="s">
-        <v>5</v>
+      <c r="G37" s="23">
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="75" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B38" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="C38" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="D38" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="E38" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="F38" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="C38" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="D38" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="E38" s="22" t="s">
-        <v>146</v>
-      </c>
-      <c r="F38" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="G38" s="24" t="s">
-        <v>10</v>
+      <c r="G38" s="24">
+        <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="45" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C39" s="25">
         <v>3000</v>
@@ -2149,108 +2137,108 @@
       <c r="F39" s="25">
         <v>2880</v>
       </c>
-      <c r="G39" s="26" t="s">
-        <v>5</v>
+      <c r="G39" s="26">
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B40" s="28" t="s">
+        <v>145</v>
+      </c>
+      <c r="C40" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="D40" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="E40" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="F40" s="29" t="s">
         <v>149</v>
       </c>
-      <c r="C40" s="29" t="s">
-        <v>150</v>
-      </c>
-      <c r="D40" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="E40" s="29" t="s">
-        <v>152</v>
-      </c>
-      <c r="F40" s="29" t="s">
-        <v>153</v>
-      </c>
-      <c r="G40" s="27" t="s">
-        <v>16</v>
+      <c r="G40" s="27">
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="120" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B41" s="20" t="s">
+        <v>150</v>
+      </c>
+      <c r="C41" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="D41" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="E41" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="F41" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="C41" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="D41" s="22" t="s">
-        <v>156</v>
-      </c>
-      <c r="E41" s="22" t="s">
-        <v>157</v>
-      </c>
-      <c r="F41" s="22" t="s">
-        <v>158</v>
-      </c>
-      <c r="G41" s="24" t="s">
-        <v>22</v>
+      <c r="G41" s="24">
+        <v>4</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B42" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="C42" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="D42" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="E42" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="F42" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="C42" s="22" t="s">
-        <v>160</v>
-      </c>
-      <c r="D42" s="22" t="s">
-        <v>161</v>
-      </c>
-      <c r="E42" s="22" t="s">
-        <v>162</v>
-      </c>
-      <c r="F42" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="G42" s="24" t="s">
-        <v>16</v>
+      <c r="G42" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B43" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="C43" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="D43" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="E43" s="25" t="s">
+        <v>163</v>
+      </c>
+      <c r="F43" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="C43" s="25" t="s">
-        <v>165</v>
-      </c>
-      <c r="D43" s="25" t="s">
-        <v>166</v>
-      </c>
-      <c r="E43" s="25" t="s">
-        <v>167</v>
-      </c>
-      <c r="F43" s="25" t="s">
-        <v>168</v>
-      </c>
-      <c r="G43" s="27" t="s">
-        <v>10</v>
+      <c r="G43" s="27">
+        <v>3</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B44" s="28" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C44" s="25">
         <v>400</v>
@@ -2264,62 +2252,62 @@
       <c r="F44" s="25">
         <v>412</v>
       </c>
-      <c r="G44" s="27" t="s">
-        <v>5</v>
+      <c r="G44" s="27">
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="45" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B45" s="28" t="s">
+        <v>166</v>
+      </c>
+      <c r="C45" s="25" t="s">
+        <v>167</v>
+      </c>
+      <c r="D45" s="25" t="s">
+        <v>168</v>
+      </c>
+      <c r="E45" s="25" t="s">
+        <v>169</v>
+      </c>
+      <c r="F45" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="C45" s="25" t="s">
-        <v>171</v>
-      </c>
-      <c r="D45" s="25" t="s">
-        <v>172</v>
-      </c>
-      <c r="E45" s="25" t="s">
-        <v>173</v>
-      </c>
-      <c r="F45" s="25" t="s">
-        <v>174</v>
-      </c>
-      <c r="G45" s="27" t="s">
-        <v>5</v>
+      <c r="G45" s="27">
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B46" s="28" t="s">
+        <v>171</v>
+      </c>
+      <c r="C46" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="D46" s="25" t="s">
+        <v>173</v>
+      </c>
+      <c r="E46" s="25" t="s">
+        <v>174</v>
+      </c>
+      <c r="F46" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="C46" s="25" t="s">
-        <v>176</v>
-      </c>
-      <c r="D46" s="25" t="s">
-        <v>177</v>
-      </c>
-      <c r="E46" s="25" t="s">
-        <v>178</v>
-      </c>
-      <c r="F46" s="25" t="s">
-        <v>179</v>
-      </c>
-      <c r="G46" s="27" t="s">
-        <v>16</v>
+      <c r="G46" s="27">
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C47" s="22">
         <v>1.1000000000000001</v>
@@ -2333,16 +2321,16 @@
       <c r="F47" s="22">
         <v>1.3</v>
       </c>
-      <c r="G47" s="30" t="s">
-        <v>16</v>
+      <c r="G47" s="30">
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C48" s="22">
         <v>1</v>
@@ -2356,215 +2344,215 @@
       <c r="F48" s="22">
         <v>1.4</v>
       </c>
-      <c r="G48" s="30" t="s">
-        <v>5</v>
+      <c r="G48" s="30">
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B49" s="28" t="s">
+        <v>178</v>
+      </c>
+      <c r="C49" s="25" t="s">
+        <v>179</v>
+      </c>
+      <c r="D49" s="25" t="s">
+        <v>180</v>
+      </c>
+      <c r="E49" s="25" t="s">
+        <v>181</v>
+      </c>
+      <c r="F49" s="25" t="s">
         <v>182</v>
       </c>
-      <c r="C49" s="25" t="s">
-        <v>183</v>
-      </c>
-      <c r="D49" s="25" t="s">
-        <v>184</v>
-      </c>
-      <c r="E49" s="25" t="s">
-        <v>185</v>
-      </c>
-      <c r="F49" s="25" t="s">
-        <v>186</v>
-      </c>
-      <c r="G49" s="24" t="s">
-        <v>16</v>
+      <c r="G49" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B50" s="28" t="s">
+        <v>183</v>
+      </c>
+      <c r="C50" s="25" t="s">
+        <v>184</v>
+      </c>
+      <c r="D50" s="25" t="s">
+        <v>185</v>
+      </c>
+      <c r="E50" s="25" t="s">
+        <v>186</v>
+      </c>
+      <c r="F50" s="25" t="s">
         <v>187</v>
       </c>
-      <c r="C50" s="25" t="s">
-        <v>188</v>
-      </c>
-      <c r="D50" s="25" t="s">
-        <v>189</v>
-      </c>
-      <c r="E50" s="25" t="s">
-        <v>190</v>
-      </c>
-      <c r="F50" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="G50" s="27" t="s">
-        <v>10</v>
+      <c r="G50" s="27">
+        <v>3</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B51" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="F51" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="C51" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="E51" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="F51" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="G51" s="10" t="s">
-        <v>10</v>
+      <c r="G51" s="10">
+        <v>3</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="60" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B52" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="F52" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="C52" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="E52" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="F52" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="G52" s="10" t="s">
-        <v>5</v>
+      <c r="G52" s="10">
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="45" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B53" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="F53" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="C53" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="E53" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="F53" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="G53" s="10" t="s">
-        <v>5</v>
+      <c r="G53" s="10">
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B54" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="C54" s="22" t="s">
+        <v>204</v>
+      </c>
+      <c r="D54" s="22" t="s">
+        <v>205</v>
+      </c>
+      <c r="E54" s="22" t="s">
+        <v>206</v>
+      </c>
+      <c r="F54" s="22" t="s">
         <v>207</v>
       </c>
-      <c r="C54" s="22" t="s">
-        <v>208</v>
-      </c>
-      <c r="D54" s="22" t="s">
-        <v>209</v>
-      </c>
-      <c r="E54" s="22" t="s">
-        <v>210</v>
-      </c>
-      <c r="F54" s="22" t="s">
-        <v>211</v>
-      </c>
-      <c r="G54" s="26" t="s">
-        <v>16</v>
+      <c r="G54" s="26">
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B55" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="C55" s="22" t="s">
+        <v>209</v>
+      </c>
+      <c r="D55" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="E55" s="22" t="s">
+        <v>211</v>
+      </c>
+      <c r="F55" s="22" t="s">
         <v>212</v>
       </c>
-      <c r="C55" s="22" t="s">
-        <v>213</v>
-      </c>
-      <c r="D55" s="22" t="s">
-        <v>214</v>
-      </c>
-      <c r="E55" s="22" t="s">
-        <v>215</v>
-      </c>
-      <c r="F55" s="22" t="s">
-        <v>216</v>
-      </c>
-      <c r="G55" s="26" t="s">
-        <v>16</v>
+      <c r="G55" s="26">
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="30" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B56" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="C56" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="D56" s="22" t="s">
+        <v>215</v>
+      </c>
+      <c r="E56" s="22" t="s">
+        <v>216</v>
+      </c>
+      <c r="F56" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="C56" s="22" t="s">
-        <v>218</v>
-      </c>
-      <c r="D56" s="22" t="s">
-        <v>219</v>
-      </c>
-      <c r="E56" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="F56" s="22" t="s">
-        <v>221</v>
-      </c>
-      <c r="G56" s="26" t="s">
-        <v>5</v>
+      <c r="G56" s="26">
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="45" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B57" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="C57" s="22" t="s">
+        <v>219</v>
+      </c>
+      <c r="D57" s="22" t="s">
+        <v>220</v>
+      </c>
+      <c r="E57" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="F57" s="22" t="s">
         <v>222</v>
       </c>
-      <c r="C57" s="22" t="s">
-        <v>223</v>
-      </c>
-      <c r="D57" s="22" t="s">
-        <v>224</v>
-      </c>
-      <c r="E57" s="22" t="s">
-        <v>225</v>
-      </c>
-      <c r="F57" s="22" t="s">
-        <v>226</v>
-      </c>
-      <c r="G57" s="26" t="s">
-        <v>5</v>
+      <c r="G57" s="26">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>